<commit_message>
Add Audit Logs viewer page
</commit_message>
<xml_diff>
--- a/assets.xlsx
+++ b/assets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7dfcb0381e2fbe2a/Desktop/IT Asset Management System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_2EEDD3AAD3E05C074113C3734B5ED87656CD7B38" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_2EEDD3AAD3E05C074113C3734B5ED87656CD7B38" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42192F63-B1A5-4B86-9D94-A81FA3D727BE}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="182">
   <si>
     <t>Assets Id</t>
   </si>
@@ -365,9 +365,6 @@
   </si>
   <si>
     <t>INV-1010</t>
-  </si>
-  <si>
-    <t>10</t>
   </si>
   <si>
     <t>TAG-010</t>
@@ -607,9 +604,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -914,6 +912,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="9" max="9" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -1463,7 +1468,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:19" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>108</v>
       </c>
@@ -1500,40 +1505,40 @@
       <c r="L11" t="s">
         <v>113</v>
       </c>
-      <c r="M11" t="s">
+      <c r="M11" s="2">
+        <v>10</v>
+      </c>
+      <c r="N11" t="s">
         <v>115</v>
-      </c>
-      <c r="N11" t="s">
-        <v>116</v>
       </c>
       <c r="O11" t="s">
         <v>30</v>
       </c>
       <c r="P11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="Q11" t="s">
         <v>31</v>
       </c>
       <c r="S11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B12" t="s">
         <v>66</v>
       </c>
       <c r="C12" t="s">
+        <v>119</v>
+      </c>
+      <c r="D12" t="s">
         <v>120</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>121</v>
-      </c>
-      <c r="E12" t="s">
-        <v>122</v>
       </c>
       <c r="F12" t="s">
         <v>70</v>
@@ -1542,7 +1547,7 @@
         <v>25</v>
       </c>
       <c r="H12" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I12" s="1">
         <v>46033</v>
@@ -1551,7 +1556,7 @@
         <v>27</v>
       </c>
       <c r="K12" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="L12" s="1">
         <v>46033</v>
@@ -1560,10 +1565,10 @@
         <v>11</v>
       </c>
       <c r="N12" t="s">
+        <v>124</v>
+      </c>
+      <c r="O12" t="s">
         <v>125</v>
-      </c>
-      <c r="O12" t="s">
-        <v>126</v>
       </c>
       <c r="P12" s="1">
         <v>46763</v>
@@ -1574,7 +1579,7 @@
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B13" t="s">
         <v>34</v>
@@ -1583,19 +1588,19 @@
         <v>76</v>
       </c>
       <c r="D13" t="s">
+        <v>127</v>
+      </c>
+      <c r="E13" t="s">
         <v>128</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>129</v>
-      </c>
-      <c r="F13" t="s">
-        <v>130</v>
       </c>
       <c r="G13" t="s">
         <v>25</v>
       </c>
       <c r="H13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I13" s="1">
         <v>46034</v>
@@ -1604,7 +1609,7 @@
         <v>39</v>
       </c>
       <c r="K13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="L13" s="1">
         <v>46034</v>
@@ -1613,10 +1618,10 @@
         <v>12</v>
       </c>
       <c r="N13" t="s">
+        <v>132</v>
+      </c>
+      <c r="O13" t="s">
         <v>133</v>
-      </c>
-      <c r="O13" t="s">
-        <v>134</v>
       </c>
       <c r="P13" s="1">
         <v>47495</v>
@@ -1627,7 +1632,7 @@
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B14" t="s">
         <v>66</v>
@@ -1636,10 +1641,10 @@
         <v>21</v>
       </c>
       <c r="D14" t="s">
+        <v>135</v>
+      </c>
+      <c r="E14" t="s">
         <v>136</v>
-      </c>
-      <c r="E14" t="s">
-        <v>137</v>
       </c>
       <c r="F14" t="s">
         <v>79</v>
@@ -1648,7 +1653,7 @@
         <v>25</v>
       </c>
       <c r="H14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I14" s="1">
         <v>46035</v>
@@ -1657,7 +1662,7 @@
         <v>50</v>
       </c>
       <c r="K14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L14" s="1">
         <v>46035</v>
@@ -1666,7 +1671,7 @@
         <v>13</v>
       </c>
       <c r="N14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="O14" t="s">
         <v>83</v>
@@ -1680,19 +1685,19 @@
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B15" t="s">
         <v>20</v>
       </c>
       <c r="C15" t="s">
+        <v>141</v>
+      </c>
+      <c r="D15" t="s">
         <v>142</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>143</v>
-      </c>
-      <c r="E15" t="s">
-        <v>144</v>
       </c>
       <c r="F15" t="s">
         <v>48</v>
@@ -1701,7 +1706,7 @@
         <v>25</v>
       </c>
       <c r="H15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I15" s="1">
         <v>46036</v>
@@ -1710,7 +1715,7 @@
         <v>61</v>
       </c>
       <c r="K15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L15" s="1">
         <v>46036</v>
@@ -1719,10 +1724,10 @@
         <v>14</v>
       </c>
       <c r="N15" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="O15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="P15" s="1">
         <v>46766</v>
@@ -1733,7 +1738,7 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B16" t="s">
         <v>44</v>
@@ -1742,10 +1747,10 @@
         <v>45</v>
       </c>
       <c r="D16" t="s">
+        <v>148</v>
+      </c>
+      <c r="E16" t="s">
         <v>149</v>
-      </c>
-      <c r="E16" t="s">
-        <v>150</v>
       </c>
       <c r="F16" t="s">
         <v>37</v>
@@ -1754,7 +1759,7 @@
         <v>111</v>
       </c>
       <c r="H16" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I16" s="1">
         <v>46037</v>
@@ -1763,7 +1768,7 @@
         <v>72</v>
       </c>
       <c r="K16" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L16" s="1">
         <v>46037</v>
@@ -1772,7 +1777,7 @@
         <v>15</v>
       </c>
       <c r="N16" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="O16" t="s">
         <v>64</v>
@@ -1786,7 +1791,7 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B17" t="s">
         <v>34</v>
@@ -1795,10 +1800,10 @@
         <v>76</v>
       </c>
       <c r="D17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E17" t="s">
         <v>155</v>
-      </c>
-      <c r="E17" t="s">
-        <v>156</v>
       </c>
       <c r="F17" t="s">
         <v>59</v>
@@ -1807,7 +1812,7 @@
         <v>25</v>
       </c>
       <c r="H17" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I17" s="1">
         <v>46038</v>
@@ -1816,7 +1821,7 @@
         <v>27</v>
       </c>
       <c r="K17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L17" s="1">
         <v>46038</v>
@@ -1825,7 +1830,7 @@
         <v>16</v>
       </c>
       <c r="N17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O17" t="s">
         <v>83</v>
@@ -1839,7 +1844,7 @@
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B18" t="s">
         <v>34</v>
@@ -1848,10 +1853,10 @@
         <v>76</v>
       </c>
       <c r="D18" t="s">
+        <v>154</v>
+      </c>
+      <c r="E18" t="s">
         <v>155</v>
-      </c>
-      <c r="E18" t="s">
-        <v>156</v>
       </c>
       <c r="F18" t="s">
         <v>59</v>
@@ -1860,7 +1865,7 @@
         <v>25</v>
       </c>
       <c r="H18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I18" s="1">
         <v>46038</v>
@@ -1869,7 +1874,7 @@
         <v>27</v>
       </c>
       <c r="K18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L18" s="1">
         <v>46039</v>
@@ -1878,7 +1883,7 @@
         <v>17</v>
       </c>
       <c r="N18" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="O18" t="s">
         <v>83</v>
@@ -1892,7 +1897,7 @@
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B19" t="s">
         <v>34</v>
@@ -1901,10 +1906,10 @@
         <v>76</v>
       </c>
       <c r="D19" t="s">
+        <v>162</v>
+      </c>
+      <c r="E19" t="s">
         <v>163</v>
-      </c>
-      <c r="E19" t="s">
-        <v>164</v>
       </c>
       <c r="F19" t="s">
         <v>24</v>
@@ -1913,7 +1918,7 @@
         <v>25</v>
       </c>
       <c r="H19" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="I19" s="1">
         <v>46040</v>
@@ -1922,7 +1927,7 @@
         <v>50</v>
       </c>
       <c r="K19" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="L19" s="1">
         <v>46040</v>
@@ -1931,7 +1936,7 @@
         <v>18</v>
       </c>
       <c r="N19" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="O19" t="s">
         <v>83</v>
@@ -1945,7 +1950,7 @@
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B20" t="s">
         <v>44</v>
@@ -1954,19 +1959,19 @@
         <v>45</v>
       </c>
       <c r="D20" t="s">
+        <v>168</v>
+      </c>
+      <c r="E20" t="s">
         <v>169</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>170</v>
-      </c>
-      <c r="F20" t="s">
-        <v>171</v>
       </c>
       <c r="G20" t="s">
         <v>25</v>
       </c>
       <c r="H20" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="I20" s="1">
         <v>46041</v>
@@ -1975,7 +1980,7 @@
         <v>61</v>
       </c>
       <c r="K20" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="L20" s="1">
         <v>46041</v>
@@ -1984,10 +1989,10 @@
         <v>19</v>
       </c>
       <c r="N20" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="O20" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="P20" s="1">
         <v>46771</v>
@@ -1998,7 +2003,7 @@
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B21" t="s">
         <v>44</v>
@@ -2010,7 +2015,7 @@
         <v>77</v>
       </c>
       <c r="E21" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F21" t="s">
         <v>59</v>
@@ -2019,37 +2024,37 @@
         <v>25</v>
       </c>
       <c r="H21" t="s">
+        <v>176</v>
+      </c>
+      <c r="I21" t="s">
         <v>177</v>
       </c>
-      <c r="I21" t="s">
+      <c r="J21" t="s">
         <v>178</v>
       </c>
-      <c r="J21" t="s">
+      <c r="K21" t="s">
         <v>179</v>
       </c>
-      <c r="K21" t="s">
-        <v>180</v>
-      </c>
       <c r="L21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="M21">
         <v>20</v>
       </c>
       <c r="N21" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="O21" t="s">
         <v>30</v>
       </c>
       <c r="P21" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q21" t="s">
         <v>31</v>
       </c>
       <c r="S21" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: stage all modified templates and requirements files
</commit_message>
<xml_diff>
--- a/assets.xlsx
+++ b/assets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7dfcb0381e2fbe2a/Desktop/IT Asset Management System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_2EEDD3AAD3E05C074113C3734B5ED87656CD7B38" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42192F63-B1A5-4B86-9D94-A81FA3D727BE}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="11_2EEDD3AAD3E05C074113C3734B5ED87656CD7B38" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50E85160-E5F5-4A60-BE64-40E757A24A60}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -604,10 +604,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -623,6 +622,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -913,6 +916,9 @@
   <dimension ref="A1:S21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="4" max="4" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.81640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.6328125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="17.54296875" bestFit="1" customWidth="1"/>
@@ -1505,7 +1511,7 @@
       <c r="L11" t="s">
         <v>113</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11">
         <v>10</v>
       </c>
       <c r="N11" t="s">

</xml_diff>